<commit_message>
locked all parameters naming cells, and allowed  user to select only values, units, and adding extra chemicals
</commit_message>
<xml_diff>
--- a/data_in_templates/input_isotherm_temp.xlsx
+++ b/data_in_templates/input_isotherm_temp.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mohammedfaran/Desktop/python_models/ReactorModels/data_in_templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A25D1E7-69D8-CA4E-A596-9A9F2EBB3A59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D20F0B6-F5F3-2040-ADA9-E6845F238388}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="940" yWindow="500" windowWidth="27860" windowHeight="17500" xr2:uid="{FB75EC0D-8373-7F4F-A4DF-7E2B42744032}"/>
   </bookViews>
@@ -295,70 +295,89 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -697,87 +716,89 @@
   <dimension ref="A1:AX17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="11.6640625" customWidth="1"/>
-    <col min="6" max="6" width="11.6640625" customWidth="1"/>
-    <col min="7" max="7" width="20.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="93" customWidth="1"/>
-    <col min="10" max="24" width="11.6640625" customWidth="1"/>
+    <col min="1" max="1" width="12.6640625" style="15" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="11.6640625" style="15" customWidth="1"/>
+    <col min="4" max="5" width="10.83203125" style="15"/>
+    <col min="6" max="6" width="11.6640625" style="15" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" style="15" customWidth="1"/>
+    <col min="8" max="8" width="12.6640625" style="15" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="93" style="15" customWidth="1"/>
+    <col min="10" max="24" width="11.6640625" style="15" customWidth="1"/>
+    <col min="25" max="16384" width="10.83203125" style="15"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:50" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="21"/>
+      <c r="B1" s="14"/>
     </row>
     <row r="2" spans="1:50" x14ac:dyDescent="0.2">
-      <c r="A2" s="7"/>
-      <c r="B2" s="9" t="s">
+      <c r="A2" s="16"/>
+      <c r="B2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="22" t="s">
+      <c r="C2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="22"/>
-      <c r="E2" s="23" t="s">
+      <c r="D2" s="3"/>
+      <c r="E2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="23"/>
-      <c r="H2" s="24" t="s">
+      <c r="F2" s="4"/>
+      <c r="H2" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="24" t="s">
+      <c r="I2" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="13"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="14"/>
-      <c r="M2" s="14"/>
-      <c r="N2" s="14"/>
-      <c r="O2" s="14"/>
-      <c r="P2" s="14"/>
-      <c r="Q2" s="14"/>
-      <c r="R2" s="14"/>
-      <c r="S2" s="14"/>
-      <c r="T2" s="14"/>
-      <c r="U2" s="14"/>
-      <c r="V2" s="14"/>
-      <c r="W2" s="14"/>
-      <c r="X2" s="14"/>
-      <c r="Y2" s="14"/>
-      <c r="Z2" s="14"/>
-      <c r="AA2" s="14"/>
-      <c r="AB2" s="14"/>
-      <c r="AC2" s="14"/>
-      <c r="AD2" s="14"/>
-      <c r="AE2" s="14"/>
-      <c r="AF2" s="14"/>
-      <c r="AG2" s="14"/>
-      <c r="AH2" s="14"/>
-      <c r="AI2" s="14"/>
-      <c r="AJ2" s="14"/>
-      <c r="AK2" s="14"/>
-      <c r="AL2" s="14"/>
-      <c r="AM2" s="14"/>
-      <c r="AN2" s="14"/>
-      <c r="AO2" s="14"/>
-      <c r="AP2" s="14"/>
-      <c r="AQ2" s="14"/>
-      <c r="AR2" s="14"/>
-      <c r="AS2" s="14"/>
-      <c r="AT2" s="14"/>
-      <c r="AU2" s="14"/>
-      <c r="AV2" s="14"/>
-      <c r="AW2" s="15"/>
-      <c r="AX2" s="15"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="18"/>
+      <c r="L2" s="18"/>
+      <c r="M2" s="18"/>
+      <c r="N2" s="18"/>
+      <c r="O2" s="18"/>
+      <c r="P2" s="18"/>
+      <c r="Q2" s="18"/>
+      <c r="R2" s="18"/>
+      <c r="S2" s="18"/>
+      <c r="T2" s="18"/>
+      <c r="U2" s="18"/>
+      <c r="V2" s="18"/>
+      <c r="W2" s="18"/>
+      <c r="X2" s="18"/>
+      <c r="Y2" s="18"/>
+      <c r="Z2" s="18"/>
+      <c r="AA2" s="18"/>
+      <c r="AB2" s="18"/>
+      <c r="AC2" s="18"/>
+      <c r="AD2" s="18"/>
+      <c r="AE2" s="18"/>
+      <c r="AF2" s="18"/>
+      <c r="AG2" s="18"/>
+      <c r="AH2" s="18"/>
+      <c r="AI2" s="18"/>
+      <c r="AJ2" s="18"/>
+      <c r="AK2" s="18"/>
+      <c r="AL2" s="18"/>
+      <c r="AM2" s="18"/>
+      <c r="AN2" s="18"/>
+      <c r="AO2" s="18"/>
+      <c r="AP2" s="18"/>
+      <c r="AQ2" s="18"/>
+      <c r="AR2" s="18"/>
+      <c r="AS2" s="18"/>
+      <c r="AT2" s="18"/>
+      <c r="AU2" s="18"/>
+      <c r="AV2" s="18"/>
+      <c r="AW2" s="19"/>
+      <c r="AX2" s="19"/>
     </row>
     <row r="3" spans="1:50" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="7" t="s">
         <v>0</v>
       </c>
       <c r="C3" s="8" t="s">
@@ -786,529 +807,530 @@
       <c r="D3" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="11" t="s">
+      <c r="E3" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="F3" s="11" t="s">
+      <c r="F3" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="25" t="s">
+      <c r="H3" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="19" t="s">
+      <c r="I3" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="J3" s="12"/>
-      <c r="K3" s="16"/>
-      <c r="L3" s="16"/>
-      <c r="M3" s="16"/>
-      <c r="N3" s="16"/>
-      <c r="O3" s="16"/>
-      <c r="P3" s="16"/>
-      <c r="Q3" s="16"/>
-      <c r="R3" s="16"/>
-      <c r="S3" s="16"/>
-      <c r="T3" s="16"/>
-      <c r="U3" s="16"/>
-      <c r="V3" s="16"/>
-      <c r="W3" s="16"/>
-      <c r="X3" s="16"/>
-      <c r="Y3" s="16"/>
-      <c r="Z3" s="16"/>
-      <c r="AA3" s="16"/>
-      <c r="AB3" s="16"/>
-      <c r="AC3" s="16"/>
-      <c r="AD3" s="16"/>
-      <c r="AE3" s="16"/>
-      <c r="AF3" s="16"/>
-      <c r="AG3" s="16"/>
-      <c r="AH3" s="16"/>
-      <c r="AI3" s="16"/>
-      <c r="AJ3" s="16"/>
-      <c r="AK3" s="16"/>
-      <c r="AL3" s="16"/>
-      <c r="AM3" s="16"/>
-      <c r="AN3" s="16"/>
-      <c r="AO3" s="16"/>
-      <c r="AP3" s="16"/>
-      <c r="AQ3" s="16"/>
-      <c r="AR3" s="16"/>
-      <c r="AS3" s="16"/>
-      <c r="AT3" s="16"/>
-      <c r="AU3" s="16"/>
-      <c r="AV3" s="16"/>
-      <c r="AW3" s="16"/>
-      <c r="AX3" s="16"/>
+      <c r="J3" s="20"/>
+      <c r="K3" s="21"/>
+      <c r="L3" s="21"/>
+      <c r="M3" s="21"/>
+      <c r="N3" s="21"/>
+      <c r="O3" s="21"/>
+      <c r="P3" s="21"/>
+      <c r="Q3" s="21"/>
+      <c r="R3" s="21"/>
+      <c r="S3" s="21"/>
+      <c r="T3" s="21"/>
+      <c r="U3" s="21"/>
+      <c r="V3" s="21"/>
+      <c r="W3" s="21"/>
+      <c r="X3" s="21"/>
+      <c r="Y3" s="21"/>
+      <c r="Z3" s="21"/>
+      <c r="AA3" s="21"/>
+      <c r="AB3" s="21"/>
+      <c r="AC3" s="21"/>
+      <c r="AD3" s="21"/>
+      <c r="AE3" s="21"/>
+      <c r="AF3" s="21"/>
+      <c r="AG3" s="21"/>
+      <c r="AH3" s="21"/>
+      <c r="AI3" s="21"/>
+      <c r="AJ3" s="21"/>
+      <c r="AK3" s="21"/>
+      <c r="AL3" s="21"/>
+      <c r="AM3" s="21"/>
+      <c r="AN3" s="21"/>
+      <c r="AO3" s="21"/>
+      <c r="AP3" s="21"/>
+      <c r="AQ3" s="21"/>
+      <c r="AR3" s="21"/>
+      <c r="AS3" s="21"/>
+      <c r="AT3" s="21"/>
+      <c r="AU3" s="21"/>
+      <c r="AV3" s="21"/>
+      <c r="AW3" s="21"/>
+      <c r="AX3" s="21"/>
     </row>
     <row r="4" spans="1:50" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="H4" s="25" t="s">
+      <c r="B4" s="23"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="H4" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="I4" s="19" t="s">
+      <c r="I4" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="J4" s="12"/>
-      <c r="K4" s="16"/>
-      <c r="L4" s="16"/>
-      <c r="M4" s="16"/>
-      <c r="N4" s="16"/>
-      <c r="O4" s="16"/>
-      <c r="P4" s="16"/>
-      <c r="Q4" s="16"/>
-      <c r="R4" s="16"/>
-      <c r="S4" s="16"/>
-      <c r="T4" s="16"/>
-      <c r="U4" s="16"/>
-      <c r="V4" s="16"/>
-      <c r="W4" s="16"/>
-      <c r="X4" s="16"/>
-      <c r="Y4" s="16"/>
-      <c r="Z4" s="16"/>
-      <c r="AA4" s="16"/>
-      <c r="AB4" s="16"/>
-      <c r="AC4" s="16"/>
-      <c r="AD4" s="16"/>
-      <c r="AE4" s="16"/>
-      <c r="AF4" s="16"/>
-      <c r="AG4" s="16"/>
-      <c r="AH4" s="16"/>
-      <c r="AI4" s="16"/>
-      <c r="AJ4" s="16"/>
-      <c r="AK4" s="16"/>
-      <c r="AL4" s="16"/>
-      <c r="AM4" s="16"/>
-      <c r="AN4" s="16"/>
-      <c r="AO4" s="16"/>
-      <c r="AP4" s="16"/>
-      <c r="AQ4" s="16"/>
-      <c r="AR4" s="16"/>
-      <c r="AS4" s="16"/>
-      <c r="AT4" s="16"/>
-      <c r="AU4" s="16"/>
-      <c r="AV4" s="16"/>
-      <c r="AW4" s="16"/>
-      <c r="AX4" s="16"/>
+      <c r="J4" s="20"/>
+      <c r="K4" s="21"/>
+      <c r="L4" s="21"/>
+      <c r="M4" s="21"/>
+      <c r="N4" s="21"/>
+      <c r="O4" s="21"/>
+      <c r="P4" s="21"/>
+      <c r="Q4" s="21"/>
+      <c r="R4" s="21"/>
+      <c r="S4" s="21"/>
+      <c r="T4" s="21"/>
+      <c r="U4" s="21"/>
+      <c r="V4" s="21"/>
+      <c r="W4" s="21"/>
+      <c r="X4" s="21"/>
+      <c r="Y4" s="21"/>
+      <c r="Z4" s="21"/>
+      <c r="AA4" s="21"/>
+      <c r="AB4" s="21"/>
+      <c r="AC4" s="21"/>
+      <c r="AD4" s="21"/>
+      <c r="AE4" s="21"/>
+      <c r="AF4" s="21"/>
+      <c r="AG4" s="21"/>
+      <c r="AH4" s="21"/>
+      <c r="AI4" s="21"/>
+      <c r="AJ4" s="21"/>
+      <c r="AK4" s="21"/>
+      <c r="AL4" s="21"/>
+      <c r="AM4" s="21"/>
+      <c r="AN4" s="21"/>
+      <c r="AO4" s="21"/>
+      <c r="AP4" s="21"/>
+      <c r="AQ4" s="21"/>
+      <c r="AR4" s="21"/>
+      <c r="AS4" s="21"/>
+      <c r="AT4" s="21"/>
+      <c r="AU4" s="21"/>
+      <c r="AV4" s="21"/>
+      <c r="AW4" s="21"/>
+      <c r="AX4" s="21"/>
     </row>
     <row r="5" spans="1:50" ht="32" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="H5" s="17" t="s">
+      <c r="B5" s="25"/>
+      <c r="C5" s="25"/>
+      <c r="D5" s="25"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
+      <c r="H5" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="I5" s="18" t="s">
+      <c r="I5" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="J5" s="12"/>
-      <c r="K5" s="16"/>
-      <c r="L5" s="16"/>
-      <c r="M5" s="16"/>
-      <c r="N5" s="16"/>
-      <c r="O5" s="16"/>
-      <c r="P5" s="16"/>
-      <c r="Q5" s="16"/>
-      <c r="R5" s="16"/>
-      <c r="S5" s="16"/>
-      <c r="T5" s="16"/>
-      <c r="U5" s="16"/>
-      <c r="V5" s="16"/>
-      <c r="W5" s="16"/>
-      <c r="X5" s="16"/>
-      <c r="Y5" s="16"/>
-      <c r="Z5" s="16"/>
-      <c r="AA5" s="16"/>
-      <c r="AB5" s="16"/>
-      <c r="AC5" s="16"/>
-      <c r="AD5" s="16"/>
-      <c r="AE5" s="16"/>
-      <c r="AF5" s="16"/>
-      <c r="AG5" s="16"/>
-      <c r="AH5" s="16"/>
-      <c r="AI5" s="16"/>
-      <c r="AJ5" s="16"/>
-      <c r="AK5" s="16"/>
-      <c r="AL5" s="16"/>
-      <c r="AM5" s="16"/>
-      <c r="AN5" s="16"/>
-      <c r="AO5" s="16"/>
-      <c r="AP5" s="16"/>
-      <c r="AQ5" s="16"/>
-      <c r="AR5" s="16"/>
-      <c r="AS5" s="16"/>
-      <c r="AT5" s="16"/>
-      <c r="AU5" s="16"/>
-      <c r="AV5" s="16"/>
-      <c r="AW5" s="16"/>
-      <c r="AX5" s="16"/>
+      <c r="J5" s="20"/>
+      <c r="K5" s="21"/>
+      <c r="L5" s="21"/>
+      <c r="M5" s="21"/>
+      <c r="N5" s="21"/>
+      <c r="O5" s="21"/>
+      <c r="P5" s="21"/>
+      <c r="Q5" s="21"/>
+      <c r="R5" s="21"/>
+      <c r="S5" s="21"/>
+      <c r="T5" s="21"/>
+      <c r="U5" s="21"/>
+      <c r="V5" s="21"/>
+      <c r="W5" s="21"/>
+      <c r="X5" s="21"/>
+      <c r="Y5" s="21"/>
+      <c r="Z5" s="21"/>
+      <c r="AA5" s="21"/>
+      <c r="AB5" s="21"/>
+      <c r="AC5" s="21"/>
+      <c r="AD5" s="21"/>
+      <c r="AE5" s="21"/>
+      <c r="AF5" s="21"/>
+      <c r="AG5" s="21"/>
+      <c r="AH5" s="21"/>
+      <c r="AI5" s="21"/>
+      <c r="AJ5" s="21"/>
+      <c r="AK5" s="21"/>
+      <c r="AL5" s="21"/>
+      <c r="AM5" s="21"/>
+      <c r="AN5" s="21"/>
+      <c r="AO5" s="21"/>
+      <c r="AP5" s="21"/>
+      <c r="AQ5" s="21"/>
+      <c r="AR5" s="21"/>
+      <c r="AS5" s="21"/>
+      <c r="AT5" s="21"/>
+      <c r="AU5" s="21"/>
+      <c r="AV5" s="21"/>
+      <c r="AW5" s="21"/>
+      <c r="AX5" s="21"/>
     </row>
     <row r="6" spans="1:50" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="H6" s="17" t="s">
+      <c r="B6" s="25"/>
+      <c r="C6" s="25"/>
+      <c r="D6" s="25"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="H6" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="I6" s="18" t="s">
+      <c r="I6" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="J6" s="12"/>
-      <c r="K6" s="16"/>
-      <c r="L6" s="16"/>
-      <c r="M6" s="16"/>
-      <c r="N6" s="16"/>
-      <c r="O6" s="16"/>
-      <c r="P6" s="16"/>
-      <c r="Q6" s="16"/>
-      <c r="R6" s="16"/>
-      <c r="S6" s="16"/>
-      <c r="T6" s="16"/>
-      <c r="U6" s="16"/>
-      <c r="V6" s="16"/>
-      <c r="W6" s="16"/>
-      <c r="X6" s="16"/>
-      <c r="Y6" s="16"/>
-      <c r="Z6" s="16"/>
-      <c r="AA6" s="16"/>
-      <c r="AB6" s="16"/>
-      <c r="AC6" s="16"/>
-      <c r="AD6" s="16"/>
-      <c r="AE6" s="16"/>
-      <c r="AF6" s="16"/>
-      <c r="AG6" s="16"/>
-      <c r="AH6" s="16"/>
-      <c r="AI6" s="16"/>
-      <c r="AJ6" s="16"/>
-      <c r="AK6" s="16"/>
-      <c r="AL6" s="16"/>
-      <c r="AM6" s="16"/>
-      <c r="AN6" s="16"/>
-      <c r="AO6" s="16"/>
-      <c r="AP6" s="16"/>
-      <c r="AQ6" s="16"/>
-      <c r="AR6" s="16"/>
-      <c r="AS6" s="16"/>
-      <c r="AT6" s="16"/>
-      <c r="AU6" s="16"/>
-      <c r="AV6" s="16"/>
-      <c r="AW6" s="16"/>
-      <c r="AX6" s="16"/>
+      <c r="J6" s="20"/>
+      <c r="K6" s="21"/>
+      <c r="L6" s="21"/>
+      <c r="M6" s="21"/>
+      <c r="N6" s="21"/>
+      <c r="O6" s="21"/>
+      <c r="P6" s="21"/>
+      <c r="Q6" s="21"/>
+      <c r="R6" s="21"/>
+      <c r="S6" s="21"/>
+      <c r="T6" s="21"/>
+      <c r="U6" s="21"/>
+      <c r="V6" s="21"/>
+      <c r="W6" s="21"/>
+      <c r="X6" s="21"/>
+      <c r="Y6" s="21"/>
+      <c r="Z6" s="21"/>
+      <c r="AA6" s="21"/>
+      <c r="AB6" s="21"/>
+      <c r="AC6" s="21"/>
+      <c r="AD6" s="21"/>
+      <c r="AE6" s="21"/>
+      <c r="AF6" s="21"/>
+      <c r="AG6" s="21"/>
+      <c r="AH6" s="21"/>
+      <c r="AI6" s="21"/>
+      <c r="AJ6" s="21"/>
+      <c r="AK6" s="21"/>
+      <c r="AL6" s="21"/>
+      <c r="AM6" s="21"/>
+      <c r="AN6" s="21"/>
+      <c r="AO6" s="21"/>
+      <c r="AP6" s="21"/>
+      <c r="AQ6" s="21"/>
+      <c r="AR6" s="21"/>
+      <c r="AS6" s="21"/>
+      <c r="AT6" s="21"/>
+      <c r="AU6" s="21"/>
+      <c r="AV6" s="21"/>
+      <c r="AW6" s="21"/>
+      <c r="AX6" s="21"/>
     </row>
     <row r="7" spans="1:50" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="H7" s="17" t="s">
+      <c r="B7" s="25"/>
+      <c r="C7" s="25"/>
+      <c r="D7" s="25"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
+      <c r="H7" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="I7" s="18" t="s">
+      <c r="I7" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="J7" s="12"/>
-      <c r="K7" s="16"/>
-      <c r="L7" s="16"/>
-      <c r="M7" s="16"/>
-      <c r="N7" s="16"/>
-      <c r="O7" s="16"/>
-      <c r="P7" s="16"/>
-      <c r="Q7" s="16"/>
-      <c r="R7" s="16"/>
-      <c r="S7" s="16"/>
-      <c r="T7" s="16"/>
-      <c r="U7" s="16"/>
-      <c r="V7" s="16"/>
-      <c r="W7" s="16"/>
-      <c r="X7" s="16"/>
-      <c r="Y7" s="16"/>
-      <c r="Z7" s="16"/>
-      <c r="AA7" s="16"/>
-      <c r="AB7" s="16"/>
-      <c r="AC7" s="16"/>
-      <c r="AD7" s="16"/>
-      <c r="AE7" s="16"/>
-      <c r="AF7" s="16"/>
-      <c r="AG7" s="16"/>
-      <c r="AH7" s="16"/>
-      <c r="AI7" s="16"/>
-      <c r="AJ7" s="16"/>
-      <c r="AK7" s="16"/>
-      <c r="AL7" s="16"/>
-      <c r="AM7" s="16"/>
-      <c r="AN7" s="16"/>
-      <c r="AO7" s="16"/>
-      <c r="AP7" s="16"/>
-      <c r="AQ7" s="16"/>
-      <c r="AR7" s="16"/>
-      <c r="AS7" s="16"/>
-      <c r="AT7" s="16"/>
-      <c r="AU7" s="16"/>
-      <c r="AV7" s="16"/>
-      <c r="AW7" s="16"/>
-      <c r="AX7" s="16"/>
+      <c r="J7" s="20"/>
+      <c r="K7" s="21"/>
+      <c r="L7" s="21"/>
+      <c r="M7" s="21"/>
+      <c r="N7" s="21"/>
+      <c r="O7" s="21"/>
+      <c r="P7" s="21"/>
+      <c r="Q7" s="21"/>
+      <c r="R7" s="21"/>
+      <c r="S7" s="21"/>
+      <c r="T7" s="21"/>
+      <c r="U7" s="21"/>
+      <c r="V7" s="21"/>
+      <c r="W7" s="21"/>
+      <c r="X7" s="21"/>
+      <c r="Y7" s="21"/>
+      <c r="Z7" s="21"/>
+      <c r="AA7" s="21"/>
+      <c r="AB7" s="21"/>
+      <c r="AC7" s="21"/>
+      <c r="AD7" s="21"/>
+      <c r="AE7" s="21"/>
+      <c r="AF7" s="21"/>
+      <c r="AG7" s="21"/>
+      <c r="AH7" s="21"/>
+      <c r="AI7" s="21"/>
+      <c r="AJ7" s="21"/>
+      <c r="AK7" s="21"/>
+      <c r="AL7" s="21"/>
+      <c r="AM7" s="21"/>
+      <c r="AN7" s="21"/>
+      <c r="AO7" s="21"/>
+      <c r="AP7" s="21"/>
+      <c r="AQ7" s="21"/>
+      <c r="AR7" s="21"/>
+      <c r="AS7" s="21"/>
+      <c r="AT7" s="21"/>
+      <c r="AU7" s="21"/>
+      <c r="AV7" s="21"/>
+      <c r="AW7" s="21"/>
+      <c r="AX7" s="21"/>
     </row>
     <row r="8" spans="1:50" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="H8" s="25" t="s">
+      <c r="B8" s="25"/>
+      <c r="C8" s="25"/>
+      <c r="D8" s="25"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
+      <c r="H8" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="I8" s="19" t="s">
+      <c r="I8" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="J8" s="12"/>
-      <c r="K8" s="16"/>
-      <c r="L8" s="16"/>
-      <c r="M8" s="16"/>
-      <c r="N8" s="16"/>
-      <c r="O8" s="16"/>
-      <c r="P8" s="16"/>
-      <c r="Q8" s="16"/>
-      <c r="R8" s="16"/>
-      <c r="S8" s="16"/>
-      <c r="T8" s="16"/>
-      <c r="U8" s="16"/>
-      <c r="V8" s="16"/>
-      <c r="W8" s="16"/>
-      <c r="X8" s="16"/>
-      <c r="Y8" s="16"/>
-      <c r="Z8" s="16"/>
-      <c r="AA8" s="16"/>
-      <c r="AB8" s="16"/>
-      <c r="AC8" s="16"/>
-      <c r="AD8" s="16"/>
-      <c r="AE8" s="16"/>
-      <c r="AF8" s="16"/>
-      <c r="AG8" s="16"/>
-      <c r="AH8" s="16"/>
-      <c r="AI8" s="16"/>
-      <c r="AJ8" s="16"/>
-      <c r="AK8" s="16"/>
-      <c r="AL8" s="16"/>
-      <c r="AM8" s="16"/>
-      <c r="AN8" s="16"/>
-      <c r="AO8" s="16"/>
-      <c r="AP8" s="16"/>
-      <c r="AQ8" s="16"/>
-      <c r="AR8" s="16"/>
-      <c r="AS8" s="16"/>
-      <c r="AT8" s="16"/>
-      <c r="AU8" s="16"/>
-      <c r="AV8" s="16"/>
-      <c r="AW8" s="16"/>
-      <c r="AX8" s="16"/>
+      <c r="J8" s="20"/>
+      <c r="K8" s="21"/>
+      <c r="L8" s="21"/>
+      <c r="M8" s="21"/>
+      <c r="N8" s="21"/>
+      <c r="O8" s="21"/>
+      <c r="P8" s="21"/>
+      <c r="Q8" s="21"/>
+      <c r="R8" s="21"/>
+      <c r="S8" s="21"/>
+      <c r="T8" s="21"/>
+      <c r="U8" s="21"/>
+      <c r="V8" s="21"/>
+      <c r="W8" s="21"/>
+      <c r="X8" s="21"/>
+      <c r="Y8" s="21"/>
+      <c r="Z8" s="21"/>
+      <c r="AA8" s="21"/>
+      <c r="AB8" s="21"/>
+      <c r="AC8" s="21"/>
+      <c r="AD8" s="21"/>
+      <c r="AE8" s="21"/>
+      <c r="AF8" s="21"/>
+      <c r="AG8" s="21"/>
+      <c r="AH8" s="21"/>
+      <c r="AI8" s="21"/>
+      <c r="AJ8" s="21"/>
+      <c r="AK8" s="21"/>
+      <c r="AL8" s="21"/>
+      <c r="AM8" s="21"/>
+      <c r="AN8" s="21"/>
+      <c r="AO8" s="21"/>
+      <c r="AP8" s="21"/>
+      <c r="AQ8" s="21"/>
+      <c r="AR8" s="21"/>
+      <c r="AS8" s="21"/>
+      <c r="AT8" s="21"/>
+      <c r="AU8" s="21"/>
+      <c r="AV8" s="21"/>
+      <c r="AW8" s="21"/>
+      <c r="AX8" s="21"/>
     </row>
     <row r="9" spans="1:50" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="H9" s="25" t="s">
+      <c r="B9" s="25"/>
+      <c r="C9" s="25"/>
+      <c r="D9" s="25"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16"/>
+      <c r="H9" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="I9" s="19" t="s">
+      <c r="I9" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="J9" s="12"/>
-      <c r="K9" s="16"/>
-      <c r="L9" s="16"/>
-      <c r="M9" s="16"/>
-      <c r="N9" s="16"/>
-      <c r="O9" s="16"/>
-      <c r="P9" s="16"/>
-      <c r="Q9" s="16"/>
-      <c r="R9" s="16"/>
-      <c r="S9" s="16"/>
-      <c r="T9" s="16"/>
-      <c r="U9" s="16"/>
-      <c r="V9" s="16"/>
-      <c r="W9" s="16"/>
-      <c r="X9" s="16"/>
-      <c r="Y9" s="16"/>
-      <c r="Z9" s="16"/>
-      <c r="AA9" s="16"/>
-      <c r="AB9" s="16"/>
-      <c r="AC9" s="16"/>
-      <c r="AD9" s="16"/>
-      <c r="AE9" s="16"/>
-      <c r="AF9" s="16"/>
-      <c r="AG9" s="16"/>
-      <c r="AH9" s="16"/>
-      <c r="AI9" s="16"/>
-      <c r="AJ9" s="16"/>
-      <c r="AK9" s="16"/>
-      <c r="AL9" s="16"/>
-      <c r="AM9" s="16"/>
-      <c r="AN9" s="16"/>
-      <c r="AO9" s="16"/>
-      <c r="AP9" s="16"/>
-      <c r="AQ9" s="16"/>
-      <c r="AR9" s="16"/>
-      <c r="AS9" s="16"/>
-      <c r="AT9" s="16"/>
-      <c r="AU9" s="16"/>
-      <c r="AV9" s="16"/>
-      <c r="AW9" s="16"/>
-      <c r="AX9" s="16"/>
+      <c r="J9" s="20"/>
+      <c r="K9" s="21"/>
+      <c r="L9" s="21"/>
+      <c r="M9" s="21"/>
+      <c r="N9" s="21"/>
+      <c r="O9" s="21"/>
+      <c r="P9" s="21"/>
+      <c r="Q9" s="21"/>
+      <c r="R9" s="21"/>
+      <c r="S9" s="21"/>
+      <c r="T9" s="21"/>
+      <c r="U9" s="21"/>
+      <c r="V9" s="21"/>
+      <c r="W9" s="21"/>
+      <c r="X9" s="21"/>
+      <c r="Y9" s="21"/>
+      <c r="Z9" s="21"/>
+      <c r="AA9" s="21"/>
+      <c r="AB9" s="21"/>
+      <c r="AC9" s="21"/>
+      <c r="AD9" s="21"/>
+      <c r="AE9" s="21"/>
+      <c r="AF9" s="21"/>
+      <c r="AG9" s="21"/>
+      <c r="AH9" s="21"/>
+      <c r="AI9" s="21"/>
+      <c r="AJ9" s="21"/>
+      <c r="AK9" s="21"/>
+      <c r="AL9" s="21"/>
+      <c r="AM9" s="21"/>
+      <c r="AN9" s="21"/>
+      <c r="AO9" s="21"/>
+      <c r="AP9" s="21"/>
+      <c r="AQ9" s="21"/>
+      <c r="AR9" s="21"/>
+      <c r="AS9" s="21"/>
+      <c r="AT9" s="21"/>
+      <c r="AU9" s="21"/>
+      <c r="AV9" s="21"/>
+      <c r="AW9" s="21"/>
+      <c r="AX9" s="21"/>
     </row>
     <row r="10" spans="1:50" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="16"/>
-      <c r="H10" s="16"/>
-      <c r="I10" s="16"/>
-      <c r="J10" s="16"/>
-      <c r="K10" s="16"/>
-      <c r="L10" s="16"/>
-      <c r="M10" s="16"/>
-      <c r="N10" s="16"/>
-      <c r="O10" s="16"/>
-      <c r="P10" s="16"/>
-      <c r="Q10" s="16"/>
-      <c r="R10" s="16"/>
-      <c r="S10" s="16"/>
-      <c r="T10" s="16"/>
-      <c r="U10" s="16"/>
-      <c r="V10" s="16"/>
-      <c r="W10" s="16"/>
-      <c r="X10" s="16"/>
-      <c r="Y10" s="16"/>
-      <c r="Z10" s="16"/>
-      <c r="AA10" s="16"/>
-      <c r="AB10" s="16"/>
-      <c r="AC10" s="16"/>
-      <c r="AD10" s="16"/>
-      <c r="AE10" s="16"/>
-      <c r="AF10" s="16"/>
-      <c r="AG10" s="16"/>
-      <c r="AH10" s="16"/>
-      <c r="AI10" s="16"/>
-      <c r="AJ10" s="16"/>
-      <c r="AK10" s="16"/>
-      <c r="AL10" s="16"/>
-      <c r="AM10" s="16"/>
-      <c r="AN10" s="16"/>
-      <c r="AO10" s="16"/>
-      <c r="AP10" s="16"/>
-      <c r="AQ10" s="16"/>
-      <c r="AR10" s="16"/>
-      <c r="AS10" s="16"/>
-      <c r="AT10" s="16"/>
-      <c r="AU10" s="16"/>
-      <c r="AV10" s="16"/>
-      <c r="AW10" s="16"/>
-      <c r="AX10" s="16"/>
+      <c r="B10" s="25"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="21"/>
+      <c r="H10" s="21"/>
+      <c r="I10" s="21"/>
+      <c r="J10" s="21"/>
+      <c r="K10" s="21"/>
+      <c r="L10" s="21"/>
+      <c r="M10" s="21"/>
+      <c r="N10" s="21"/>
+      <c r="O10" s="21"/>
+      <c r="P10" s="21"/>
+      <c r="Q10" s="21"/>
+      <c r="R10" s="21"/>
+      <c r="S10" s="21"/>
+      <c r="T10" s="21"/>
+      <c r="U10" s="21"/>
+      <c r="V10" s="21"/>
+      <c r="W10" s="21"/>
+      <c r="X10" s="21"/>
+      <c r="Y10" s="21"/>
+      <c r="Z10" s="21"/>
+      <c r="AA10" s="21"/>
+      <c r="AB10" s="21"/>
+      <c r="AC10" s="21"/>
+      <c r="AD10" s="21"/>
+      <c r="AE10" s="21"/>
+      <c r="AF10" s="21"/>
+      <c r="AG10" s="21"/>
+      <c r="AH10" s="21"/>
+      <c r="AI10" s="21"/>
+      <c r="AJ10" s="21"/>
+      <c r="AK10" s="21"/>
+      <c r="AL10" s="21"/>
+      <c r="AM10" s="21"/>
+      <c r="AN10" s="21"/>
+      <c r="AO10" s="21"/>
+      <c r="AP10" s="21"/>
+      <c r="AQ10" s="21"/>
+      <c r="AR10" s="21"/>
+      <c r="AS10" s="21"/>
+      <c r="AT10" s="21"/>
+      <c r="AU10" s="21"/>
+      <c r="AV10" s="21"/>
+      <c r="AW10" s="21"/>
+      <c r="AX10" s="21"/>
     </row>
     <row r="15" spans="1:50" x14ac:dyDescent="0.2">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
-      <c r="J15" s="1"/>
-      <c r="K15" s="1"/>
-      <c r="L15" s="1"/>
-      <c r="M15" s="1"/>
-      <c r="N15" s="1"/>
-      <c r="O15" s="1"/>
-      <c r="P15" s="1"/>
-      <c r="Q15" s="1"/>
-      <c r="R15" s="1"/>
-      <c r="S15" s="1"/>
-      <c r="T15" s="1"/>
-      <c r="U15" s="1"/>
-      <c r="V15" s="1"/>
-      <c r="W15" s="1"/>
-      <c r="X15" s="1"/>
+      <c r="A15" s="26"/>
+      <c r="B15" s="26"/>
+      <c r="C15" s="26"/>
+      <c r="F15" s="26"/>
+      <c r="G15" s="26"/>
+      <c r="H15" s="26"/>
+      <c r="I15" s="26"/>
+      <c r="J15" s="26"/>
+      <c r="K15" s="26"/>
+      <c r="L15" s="26"/>
+      <c r="M15" s="26"/>
+      <c r="N15" s="26"/>
+      <c r="O15" s="26"/>
+      <c r="P15" s="26"/>
+      <c r="Q15" s="26"/>
+      <c r="R15" s="26"/>
+      <c r="S15" s="26"/>
+      <c r="T15" s="26"/>
+      <c r="U15" s="26"/>
+      <c r="V15" s="26"/>
+      <c r="W15" s="26"/>
+      <c r="X15" s="26"/>
     </row>
     <row r="16" spans="1:50" x14ac:dyDescent="0.2">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
-      <c r="J16" s="1"/>
-      <c r="K16" s="1"/>
-      <c r="L16" s="1"/>
-      <c r="M16" s="1"/>
-      <c r="N16" s="1"/>
-      <c r="O16" s="1"/>
-      <c r="P16" s="1"/>
-      <c r="Q16" s="1"/>
-      <c r="R16" s="1"/>
-      <c r="S16" s="1"/>
-      <c r="T16" s="1"/>
-      <c r="U16" s="1"/>
-      <c r="V16" s="1"/>
-      <c r="W16" s="1"/>
-      <c r="X16" s="1"/>
+      <c r="A16" s="26"/>
+      <c r="B16" s="26"/>
+      <c r="C16" s="26"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="26"/>
+      <c r="H16" s="26"/>
+      <c r="I16" s="26"/>
+      <c r="J16" s="26"/>
+      <c r="K16" s="26"/>
+      <c r="L16" s="26"/>
+      <c r="M16" s="26"/>
+      <c r="N16" s="26"/>
+      <c r="O16" s="26"/>
+      <c r="P16" s="26"/>
+      <c r="Q16" s="26"/>
+      <c r="R16" s="26"/>
+      <c r="S16" s="26"/>
+      <c r="T16" s="26"/>
+      <c r="U16" s="26"/>
+      <c r="V16" s="26"/>
+      <c r="W16" s="26"/>
+      <c r="X16" s="26"/>
     </row>
     <row r="17" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
-      <c r="K17" s="1"/>
-      <c r="L17" s="1"/>
-      <c r="M17" s="1"/>
-      <c r="N17" s="1"/>
-      <c r="O17" s="1"/>
-      <c r="P17" s="1"/>
-      <c r="Q17" s="1"/>
-      <c r="R17" s="1"/>
-      <c r="S17" s="1"/>
-      <c r="T17" s="1"/>
-      <c r="U17" s="1"/>
-      <c r="V17" s="1"/>
-      <c r="W17" s="1"/>
-      <c r="X17" s="1"/>
+      <c r="A17" s="26"/>
+      <c r="B17" s="26"/>
+      <c r="C17" s="26"/>
+      <c r="F17" s="26"/>
+      <c r="G17" s="26"/>
+      <c r="H17" s="26"/>
+      <c r="I17" s="26"/>
+      <c r="J17" s="26"/>
+      <c r="K17" s="26"/>
+      <c r="L17" s="26"/>
+      <c r="M17" s="26"/>
+      <c r="N17" s="26"/>
+      <c r="O17" s="26"/>
+      <c r="P17" s="26"/>
+      <c r="Q17" s="26"/>
+      <c r="R17" s="26"/>
+      <c r="S17" s="26"/>
+      <c r="T17" s="26"/>
+      <c r="U17" s="26"/>
+      <c r="V17" s="26"/>
+      <c r="W17" s="26"/>
+      <c r="X17" s="26"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <mergeCells count="184">
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="E2:F2"/>

</xml_diff>